<commit_message>
Updated code for market place
</commit_message>
<xml_diff>
--- a/data/cy2027/DrugData.xlsx
+++ b/data/cy2027/DrugData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://molinahealthcare-my.sharepoint.com/personal/naresh_jangid_molinahealthcare_com/Documents/Automation/molina_automation/PlanMaterialAutomation/data/cy2027/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="19" documentId="11_7DAFE29BB6EB7810BCA00C6A4016A4F540A67422" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5A2584BA-EF8E-42A6-9B23-04C963FE3E56}"/>
+  <xr:revisionPtr revIDLastSave="20" documentId="11_7DAFE29BB6EB7810BCA00C6A4016A4F540A67422" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AB2C0E65-EBB7-474B-9199-7EB3D40949F4}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2201,7 +2201,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -2224,7 +2224,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>587</v>
       </c>
@@ -2247,7 +2247,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>587</v>
       </c>
@@ -2270,7 +2270,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>587</v>
       </c>
@@ -2293,7 +2293,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="6" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>587</v>
       </c>
@@ -3121,7 +3121,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>7</v>
       </c>
@@ -3144,7 +3144,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="43" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>587</v>
       </c>
@@ -3167,7 +3167,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="44" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>587</v>
       </c>
@@ -3190,7 +3190,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="45" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>587</v>
       </c>
@@ -3213,7 +3213,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="46" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>587</v>
       </c>
@@ -4041,7 +4041,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>7</v>
       </c>
@@ -4064,7 +4064,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="83" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>587</v>
       </c>
@@ -4087,7 +4087,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="84" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>587</v>
       </c>
@@ -4110,7 +4110,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="85" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>587</v>
       </c>
@@ -4133,7 +4133,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="86" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>587</v>
       </c>
@@ -4961,7 +4961,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="122" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
         <v>7</v>
       </c>
@@ -4984,7 +4984,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="123" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
         <v>587</v>
       </c>
@@ -5007,7 +5007,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="124" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
         <v>587</v>
       </c>
@@ -5030,7 +5030,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="125" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
         <v>587</v>
       </c>
@@ -5053,7 +5053,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="126" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
         <v>587</v>
       </c>
@@ -5881,7 +5881,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="162" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A162" t="s">
         <v>7</v>
       </c>
@@ -5904,7 +5904,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="163" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A163" t="s">
         <v>587</v>
       </c>
@@ -5927,7 +5927,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="164" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A164" t="s">
         <v>587</v>
       </c>
@@ -5950,7 +5950,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="165" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A165" t="s">
         <v>587</v>
       </c>
@@ -5973,7 +5973,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="166" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A166" t="s">
         <v>587</v>
       </c>
@@ -6801,7 +6801,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="202" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A202" t="s">
         <v>7</v>
       </c>
@@ -6824,7 +6824,7 @@
         <v>251</v>
       </c>
     </row>
-    <row r="203" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A203" t="s">
         <v>587</v>
       </c>
@@ -6847,7 +6847,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="204" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A204" t="s">
         <v>587</v>
       </c>
@@ -6870,7 +6870,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="205" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A205" t="s">
         <v>587</v>
       </c>
@@ -6893,7 +6893,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="206" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A206" t="s">
         <v>587</v>
       </c>
@@ -7721,7 +7721,7 @@
         <v>283</v>
       </c>
     </row>
-    <row r="242" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="242" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A242" t="s">
         <v>7</v>
       </c>
@@ -7744,7 +7744,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="243" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="243" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A243" t="s">
         <v>587</v>
       </c>
@@ -7767,7 +7767,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="244" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="244" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A244" t="s">
         <v>587</v>
       </c>
@@ -7790,7 +7790,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="245" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="245" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A245" t="s">
         <v>587</v>
       </c>
@@ -7813,7 +7813,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="246" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="246" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A246" t="s">
         <v>587</v>
       </c>
@@ -8641,7 +8641,7 @@
         <v>318</v>
       </c>
     </row>
-    <row r="282" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="282" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A282" t="s">
         <v>7</v>
       </c>
@@ -8664,7 +8664,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="283" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="283" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A283" t="s">
         <v>587</v>
       </c>
@@ -8687,7 +8687,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="284" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="284" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A284" t="s">
         <v>587</v>
       </c>
@@ -8710,7 +8710,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="285" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="285" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A285" t="s">
         <v>587</v>
       </c>
@@ -8733,7 +8733,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="286" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="286" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A286" t="s">
         <v>587</v>
       </c>
@@ -9561,7 +9561,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="322" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="322" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A322" t="s">
         <v>7</v>
       </c>
@@ -9584,7 +9584,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="323" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="323" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A323" t="s">
         <v>587</v>
       </c>
@@ -9607,7 +9607,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="324" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="324" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A324" t="s">
         <v>587</v>
       </c>
@@ -9630,7 +9630,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="325" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="325" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A325" t="s">
         <v>587</v>
       </c>
@@ -9653,7 +9653,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="326" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="326" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A326" t="s">
         <v>587</v>
       </c>
@@ -10481,7 +10481,7 @@
         <v>388</v>
       </c>
     </row>
-    <row r="362" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="362" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A362" t="s">
         <v>7</v>
       </c>
@@ -10504,7 +10504,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="363" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="363" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A363" t="s">
         <v>587</v>
       </c>
@@ -10527,7 +10527,7 @@
         <v>393</v>
       </c>
     </row>
-    <row r="364" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="364" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A364" t="s">
         <v>587</v>
       </c>
@@ -10550,7 +10550,7 @@
         <v>393</v>
       </c>
     </row>
-    <row r="365" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="365" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A365" t="s">
         <v>587</v>
       </c>
@@ -10573,7 +10573,7 @@
         <v>393</v>
       </c>
     </row>
-    <row r="366" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="366" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A366" t="s">
         <v>587</v>
       </c>
@@ -11401,7 +11401,7 @@
         <v>423</v>
       </c>
     </row>
-    <row r="402" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="402" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A402" t="s">
         <v>7</v>
       </c>
@@ -11424,7 +11424,7 @@
         <v>426</v>
       </c>
     </row>
-    <row r="403" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="403" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A403" t="s">
         <v>587</v>
       </c>
@@ -11447,7 +11447,7 @@
         <v>428</v>
       </c>
     </row>
-    <row r="404" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="404" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A404" t="s">
         <v>587</v>
       </c>
@@ -11470,7 +11470,7 @@
         <v>428</v>
       </c>
     </row>
-    <row r="405" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="405" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A405" t="s">
         <v>587</v>
       </c>
@@ -11493,7 +11493,7 @@
         <v>428</v>
       </c>
     </row>
-    <row r="406" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="406" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A406" t="s">
         <v>587</v>
       </c>
@@ -12321,7 +12321,7 @@
         <v>458</v>
       </c>
     </row>
-    <row r="442" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="442" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A442" t="s">
         <v>7</v>
       </c>
@@ -12344,7 +12344,7 @@
         <v>461</v>
       </c>
     </row>
-    <row r="443" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="443" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A443" t="s">
         <v>587</v>
       </c>
@@ -12367,7 +12367,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="444" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="444" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A444" t="s">
         <v>587</v>
       </c>
@@ -12390,7 +12390,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="445" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="445" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A445" t="s">
         <v>587</v>
       </c>
@@ -12413,7 +12413,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="446" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="446" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A446" t="s">
         <v>587</v>
       </c>
@@ -13241,7 +13241,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="482" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="482" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A482" t="s">
         <v>7</v>
       </c>
@@ -13264,7 +13264,7 @@
         <v>496</v>
       </c>
     </row>
-    <row r="483" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="483" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A483" t="s">
         <v>587</v>
       </c>
@@ -13287,7 +13287,7 @@
         <v>498</v>
       </c>
     </row>
-    <row r="484" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="484" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A484" t="s">
         <v>587</v>
       </c>
@@ -13310,7 +13310,7 @@
         <v>498</v>
       </c>
     </row>
-    <row r="485" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="485" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A485" t="s">
         <v>587</v>
       </c>
@@ -13333,7 +13333,7 @@
         <v>498</v>
       </c>
     </row>
-    <row r="486" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="486" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A486" t="s">
         <v>587</v>
       </c>
@@ -14161,7 +14161,7 @@
         <v>528</v>
       </c>
     </row>
-    <row r="522" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="522" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A522" t="s">
         <v>7</v>
       </c>
@@ -14184,7 +14184,7 @@
         <v>531</v>
       </c>
     </row>
-    <row r="523" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="523" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A523" t="s">
         <v>587</v>
       </c>
@@ -14207,7 +14207,7 @@
         <v>533</v>
       </c>
     </row>
-    <row r="524" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="524" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A524" t="s">
         <v>587</v>
       </c>
@@ -14230,7 +14230,7 @@
         <v>534</v>
       </c>
     </row>
-    <row r="525" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="525" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A525" t="s">
         <v>587</v>
       </c>
@@ -14253,7 +14253,7 @@
         <v>535</v>
       </c>
     </row>
-    <row r="526" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="526" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A526" t="s">
         <v>587</v>
       </c>
@@ -15085,7 +15085,7 @@
   <autoFilter ref="A1:G561" xr:uid="{00000000-0001-0000-0000-000000000000}">
     <filterColumn colId="2">
       <filters>
-        <filter val="AZ"/>
+        <filter val="CA"/>
       </filters>
     </filterColumn>
   </autoFilter>
@@ -15094,4 +15094,10 @@
     <ignoredError sqref="A1:G1 B3:G561 B2:G2" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{5e625f8d-0b53-4f56-9e46-19fa14bb2e5c}" enabled="0" method="" siteId="{5e625f8d-0b53-4f56-9e46-19fa14bb2e5c}" removed="1"/>
+</clbl:labelList>
 </file>
</xml_diff>